<commit_message>
refactor(excel): update complex formula to array in Formula_Sheet (#9)
- updated complex formula as array in Formula_Sheet to prevent errors when copying
</commit_message>
<xml_diff>
--- a/template/CheQ_Website_Production_Lighthouse Report_Template_08222025_v2.3.xlsx
+++ b/template/CheQ_Website_Production_Lighthouse Report_Template_08222025_v2.3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VonWebsterDLabajo\VS Code\Private-Lighthouse-Automation\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEA9A5D7-0EB1-42EB-9E4F-C03B481E3358}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{010A4D14-F4A1-4D1B-945F-5102D98F5F67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A3D68101-3EA1-4AB8-9C35-12A619CAE77F}"/>
   </bookViews>
@@ -1135,6 +1135,40 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="20" fontId="7" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="20" fontId="7" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="7" fillId="5" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1144,29 +1178,38 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="21" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1180,44 +1223,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="21" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1255,23 +1265,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="7" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="20" fontId="7" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="7" fillId="5" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="48">
+  <dxfs count="24">
     <dxf>
       <fill>
         <patternFill>
@@ -1470,246 +1470,6 @@
       </font>
       <fill>
         <patternFill patternType="none"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
       </fill>
     </dxf>
   </dxfs>
@@ -2062,22 +1822,22 @@
   <sheetData>
     <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D2" s="66" t="s">
+      <c r="D2" s="65" t="s">
         <v>89</v>
       </c>
-      <c r="E2" s="67"/>
+      <c r="E2" s="66"/>
       <c r="F2" s="6"/>
     </row>
     <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4"/>
-      <c r="B3" s="68" t="s">
+      <c r="B3" s="67" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="69"/>
-      <c r="D3" s="70" t="s">
-        <v>0</v>
-      </c>
-      <c r="E3" s="71"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="70"/>
       <c r="F3" s="6"/>
     </row>
     <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2107,10 +1867,10 @@
     <row r="6" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
-      <c r="D6" s="102"/>
-      <c r="E6" s="102"/>
+      <c r="D6" s="61"/>
+      <c r="E6" s="61"/>
       <c r="F6" s="6"/>
-      <c r="G6" s="61" t="str">
+      <c r="G6" s="73" t="str">
         <f>IF(OR(ISBLANK(D6),ISBLANK(E6),TEXT(D6,"mmmm d, yyyy, h:mm:ss am/pm")&lt;&gt;D6,TEXT(E6,"mmmm d, yyyy, h:mm:ss am/pm")&lt;&gt;E6),
 "Kindly add Analysis Timestamp!",
 IF(OR(Formula_Sheet!K6=0,Formula_Sheet!N6=0),
@@ -2123,7 +1883,7 @@
       </c>
     </row>
     <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="64" t="s">
+      <c r="B7" s="71" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="9" t="s">
@@ -2132,33 +1892,33 @@
       <c r="D7" s="43"/>
       <c r="E7" s="43"/>
       <c r="F7" s="6"/>
-      <c r="G7" s="62"/>
+      <c r="G7" s="74"/>
     </row>
     <row r="8" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="65"/>
+      <c r="B8" s="72"/>
       <c r="C8" s="10" t="s">
         <v>15</v>
       </c>
       <c r="D8" s="43"/>
       <c r="E8" s="43"/>
       <c r="F8" s="6"/>
-      <c r="G8" s="63"/>
+      <c r="G8" s="75"/>
     </row>
     <row r="9" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="5"/>
       <c r="C9" s="6"/>
-      <c r="D9" s="103"/>
-      <c r="E9" s="103"/>
+      <c r="D9" s="62"/>
+      <c r="E9" s="62"/>
       <c r="F9" s="6"/>
       <c r="G9" s="6"/>
     </row>
     <row r="10" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
-      <c r="D10" s="102"/>
-      <c r="E10" s="102"/>
+      <c r="D10" s="61"/>
+      <c r="E10" s="61"/>
       <c r="F10" s="6"/>
-      <c r="G10" s="61" t="str">
+      <c r="G10" s="73" t="str">
         <f>IF(OR(ISBLANK(D10),ISBLANK(E10),TEXT(D10,"mmmm d, yyyy, h:mm:ss am/pm")&lt;&gt;D10,TEXT(E10,"mmmm d, yyyy, h:mm:ss am/pm")&lt;&gt;E10),
 "Kindly add Analysis Timestamp!",
 IF(OR(Formula_Sheet!K10=0,Formula_Sheet!N10=0),
@@ -2171,7 +1931,7 @@
       </c>
     </row>
     <row r="11" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="64" t="s">
+      <c r="B11" s="71" t="s">
         <v>16</v>
       </c>
       <c r="C11" s="9" t="s">
@@ -2179,17 +1939,17 @@
       </c>
       <c r="D11" s="43"/>
       <c r="E11" s="43"/>
-      <c r="G11" s="62"/>
+      <c r="G11" s="74"/>
     </row>
     <row r="12" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="65"/>
+      <c r="B12" s="72"/>
       <c r="C12" s="10" t="s">
         <v>15</v>
       </c>
       <c r="D12" s="43"/>
       <c r="E12" s="43"/>
       <c r="F12" s="6"/>
-      <c r="G12" s="63"/>
+      <c r="G12" s="75"/>
     </row>
     <row r="13" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="5"/>
@@ -2202,10 +1962,10 @@
     <row r="14" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
-      <c r="D14" s="102"/>
-      <c r="E14" s="102"/>
+      <c r="D14" s="61"/>
+      <c r="E14" s="61"/>
       <c r="F14" s="6"/>
-      <c r="G14" s="61" t="str">
+      <c r="G14" s="73" t="str">
         <f>IF(OR(ISBLANK(D14),ISBLANK(E14),TEXT(D14,"mmmm d, yyyy, h:mm:ss am/pm")&lt;&gt;D14,TEXT(E14,"mmmm d, yyyy, h:mm:ss am/pm")&lt;&gt;E14),
 "Kindly add Analysis Timestamp!",
 IF(OR(Formula_Sheet!K14=0,Formula_Sheet!N14=0),
@@ -2218,7 +1978,7 @@
       </c>
     </row>
     <row r="15" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="64" t="s">
+      <c r="B15" s="71" t="s">
         <v>17</v>
       </c>
       <c r="C15" s="9" t="s">
@@ -2227,17 +1987,17 @@
       <c r="D15" s="43"/>
       <c r="E15" s="43"/>
       <c r="F15" s="6"/>
-      <c r="G15" s="62"/>
+      <c r="G15" s="74"/>
     </row>
     <row r="16" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="65"/>
+      <c r="B16" s="72"/>
       <c r="C16" s="10" t="s">
         <v>15</v>
       </c>
       <c r="D16" s="43"/>
       <c r="E16" s="43"/>
       <c r="F16" s="6"/>
-      <c r="G16" s="63"/>
+      <c r="G16" s="75"/>
     </row>
     <row r="17" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="5"/>
@@ -2250,10 +2010,10 @@
     <row r="18" spans="2:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
-      <c r="D18" s="104"/>
-      <c r="E18" s="102"/>
+      <c r="D18" s="63"/>
+      <c r="E18" s="61"/>
       <c r="F18" s="6"/>
-      <c r="G18" s="61" t="str">
+      <c r="G18" s="73" t="str">
         <f>IF(OR(ISBLANK(D18),ISBLANK(E18),TEXT(D18,"mmmm d, yyyy, h:mm:ss am/pm")&lt;&gt;D18,TEXT(E18,"mmmm d, yyyy, h:mm:ss am/pm")&lt;&gt;E18),
 "Kindly add Analysis Timestamp!",
 IF(OR(Formula_Sheet!K18=0,Formula_Sheet!N18=0),
@@ -2266,7 +2026,7 @@
       </c>
     </row>
     <row r="19" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="64" t="s">
+      <c r="B19" s="71" t="s">
         <v>18</v>
       </c>
       <c r="C19" s="9" t="s">
@@ -2275,17 +2035,17 @@
       <c r="D19" s="43"/>
       <c r="E19" s="43"/>
       <c r="F19" s="6"/>
-      <c r="G19" s="62"/>
+      <c r="G19" s="74"/>
     </row>
     <row r="20" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="65"/>
+      <c r="B20" s="72"/>
       <c r="C20" s="10" t="s">
         <v>15</v>
       </c>
       <c r="D20" s="43"/>
       <c r="E20" s="43"/>
       <c r="F20" s="6"/>
-      <c r="G20" s="63"/>
+      <c r="G20" s="75"/>
     </row>
     <row r="21" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="5"/>
@@ -2298,10 +2058,10 @@
     <row r="22" spans="2:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
-      <c r="D22" s="102"/>
-      <c r="E22" s="102"/>
+      <c r="D22" s="61"/>
+      <c r="E22" s="61"/>
       <c r="F22" s="6"/>
-      <c r="G22" s="61" t="str">
+      <c r="G22" s="73" t="str">
         <f>IF(OR(ISBLANK(D22),ISBLANK(E22),TEXT(D22,"mmmm d, yyyy, h:mm:ss am/pm")&lt;&gt;D22,TEXT(E22,"mmmm d, yyyy, h:mm:ss am/pm")&lt;&gt;E22),
 "Kindly add Analysis Timestamp!",
 IF(OR(Formula_Sheet!K22=0,Formula_Sheet!N22=0),
@@ -2314,7 +2074,7 @@
       </c>
     </row>
     <row r="23" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="64" t="s">
+      <c r="B23" s="71" t="s">
         <v>19</v>
       </c>
       <c r="C23" s="9" t="s">
@@ -2323,33 +2083,33 @@
       <c r="D23" s="43"/>
       <c r="E23" s="43"/>
       <c r="F23" s="6"/>
-      <c r="G23" s="62"/>
+      <c r="G23" s="74"/>
     </row>
     <row r="24" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="65"/>
+      <c r="B24" s="72"/>
       <c r="C24" s="10" t="s">
         <v>15</v>
       </c>
       <c r="D24" s="43"/>
       <c r="E24" s="43"/>
       <c r="F24" s="6"/>
-      <c r="G24" s="63"/>
+      <c r="G24" s="75"/>
     </row>
     <row r="25" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="5"/>
       <c r="C25" s="6"/>
       <c r="D25" s="42"/>
-      <c r="E25" s="105"/>
+      <c r="E25" s="64"/>
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
     </row>
     <row r="26" spans="2:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
-      <c r="D26" s="102"/>
-      <c r="E26" s="102"/>
+      <c r="D26" s="61"/>
+      <c r="E26" s="61"/>
       <c r="F26" s="6"/>
-      <c r="G26" s="61" t="str">
+      <c r="G26" s="73" t="str">
         <f>IF(OR(ISBLANK(D26),ISBLANK(E26),TEXT(D26,"mmmm d, yyyy, h:mm:ss am/pm")&lt;&gt;D26,TEXT(E26,"mmmm d, yyyy, h:mm:ss am/pm")&lt;&gt;E26),
 "Kindly add Analysis Timestamp!",
 IF(OR(Formula_Sheet!K26=0,Formula_Sheet!N26=0),
@@ -2362,7 +2122,7 @@
       </c>
     </row>
     <row r="27" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="64" t="s">
+      <c r="B27" s="71" t="s">
         <v>20</v>
       </c>
       <c r="C27" s="9" t="s">
@@ -2371,17 +2131,17 @@
       <c r="D27" s="43"/>
       <c r="E27" s="43"/>
       <c r="F27" s="6"/>
-      <c r="G27" s="62"/>
+      <c r="G27" s="74"/>
     </row>
     <row r="28" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="65"/>
+      <c r="B28" s="72"/>
       <c r="C28" s="10" t="s">
         <v>15</v>
       </c>
       <c r="D28" s="43"/>
       <c r="E28" s="43"/>
       <c r="F28" s="6"/>
-      <c r="G28" s="63"/>
+      <c r="G28" s="75"/>
     </row>
     <row r="29" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B29" s="5"/>
@@ -2394,10 +2154,10 @@
     <row r="30" spans="2:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>
-      <c r="D30" s="102"/>
-      <c r="E30" s="104"/>
+      <c r="D30" s="61"/>
+      <c r="E30" s="63"/>
       <c r="F30" s="6"/>
-      <c r="G30" s="61" t="str">
+      <c r="G30" s="73" t="str">
         <f>IF(OR(ISBLANK(D30),ISBLANK(E30),TEXT(D30,"mmmm d, yyyy, h:mm:ss am/pm")&lt;&gt;D30,TEXT(E30,"mmmm d, yyyy, h:mm:ss am/pm")&lt;&gt;E30),
 "Kindly add Analysis Timestamp!",
 IF(OR(Formula_Sheet!K30=0,Formula_Sheet!N30=0),
@@ -2410,7 +2170,7 @@
       </c>
     </row>
     <row r="31" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="64" t="s">
+      <c r="B31" s="71" t="s">
         <v>21</v>
       </c>
       <c r="C31" s="9" t="s">
@@ -2419,17 +2179,17 @@
       <c r="D31" s="43"/>
       <c r="E31" s="43"/>
       <c r="F31" s="6"/>
-      <c r="G31" s="62"/>
+      <c r="G31" s="74"/>
     </row>
     <row r="32" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="65"/>
+      <c r="B32" s="72"/>
       <c r="C32" s="10" t="s">
         <v>15</v>
       </c>
       <c r="D32" s="43"/>
       <c r="E32" s="43"/>
       <c r="F32" s="6"/>
-      <c r="G32" s="63"/>
+      <c r="G32" s="75"/>
     </row>
     <row r="33" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B33" s="5"/>
@@ -2442,10 +2202,10 @@
     <row r="34" spans="2:7" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
-      <c r="D34" s="102"/>
-      <c r="E34" s="104"/>
+      <c r="D34" s="61"/>
+      <c r="E34" s="63"/>
       <c r="F34" s="6"/>
-      <c r="G34" s="61" t="str">
+      <c r="G34" s="73" t="str">
         <f>IF(OR(ISBLANK(D34),ISBLANK(E34),TEXT(D34,"mmmm d, yyyy, h:mm:ss am/pm")&lt;&gt;D34,TEXT(E34,"mmmm d, yyyy, h:mm:ss am/pm")&lt;&gt;E34),
 "Kindly add Analysis Timestamp!",
 IF(OR(Formula_Sheet!K34=0,Formula_Sheet!N34=0),
@@ -2458,7 +2218,7 @@
       </c>
     </row>
     <row r="35" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="64" t="s">
+      <c r="B35" s="71" t="s">
         <v>22</v>
       </c>
       <c r="C35" s="9" t="s">
@@ -2467,17 +2227,17 @@
       <c r="D35" s="43"/>
       <c r="E35" s="43"/>
       <c r="F35" s="6"/>
-      <c r="G35" s="62"/>
+      <c r="G35" s="74"/>
     </row>
     <row r="36" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="65"/>
+      <c r="B36" s="72"/>
       <c r="C36" s="10" t="s">
         <v>15</v>
       </c>
       <c r="D36" s="43"/>
       <c r="E36" s="43"/>
       <c r="F36" s="6"/>
-      <c r="G36" s="63"/>
+      <c r="G36" s="75"/>
     </row>
     <row r="37" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C37" s="6"/>
@@ -2493,7 +2253,7 @@
         <v>24</v>
       </c>
       <c r="F38" s="6"/>
-      <c r="G38" s="61" t="str">
+      <c r="G38" s="73" t="str">
         <f>IF(OR(Formula_Sheet!J39=0,Formula_Sheet!K39=0),
 "Kindly, fill the Performance Score first!",
 Formula_Sheet!T61 &amp; Formula_Sheet!T62 &amp;
@@ -2515,7 +2275,7 @@
         <v>27</v>
       </c>
       <c r="F39" s="6"/>
-      <c r="G39" s="62"/>
+      <c r="G39" s="74"/>
     </row>
     <row r="40" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C40" s="13" t="s">
@@ -2525,21 +2285,16 @@
         <v>30</v>
       </c>
       <c r="F40" s="6"/>
-      <c r="G40" s="62"/>
+      <c r="G40" s="74"/>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="G41" s="62"/>
+      <c r="G41" s="74"/>
     </row>
     <row r="42" spans="2:7" ht="64.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="G42" s="63"/>
+      <c r="G42" s="75"/>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="B11:B12"/>
     <mergeCell ref="G6:G8"/>
     <mergeCell ref="G18:G20"/>
     <mergeCell ref="G38:G42"/>
@@ -2555,6 +2310,11 @@
     <mergeCell ref="B27:B28"/>
     <mergeCell ref="G14:G16"/>
     <mergeCell ref="G10:G12"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="B11:B12"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:E8">
     <cfRule type="cellIs" dxfId="23" priority="4" operator="lessThan">
@@ -2694,31 +2454,31 @@
       <c r="J3" s="31"/>
     </row>
     <row r="4" spans="9:40" x14ac:dyDescent="0.3">
-      <c r="T4" s="90" t="s">
+      <c r="T4" s="94" t="s">
         <v>54</v>
       </c>
-      <c r="U4" s="91"/>
-      <c r="V4" s="91"/>
-      <c r="W4" s="91"/>
-      <c r="X4" s="91"/>
-      <c r="Y4" s="91"/>
-      <c r="Z4" s="91"/>
-      <c r="AA4" s="91"/>
-      <c r="AB4" s="92"/>
+      <c r="U4" s="95"/>
+      <c r="V4" s="95"/>
+      <c r="W4" s="95"/>
+      <c r="X4" s="95"/>
+      <c r="Y4" s="95"/>
+      <c r="Z4" s="95"/>
+      <c r="AA4" s="95"/>
+      <c r="AB4" s="96"/>
       <c r="AC4" s="44"/>
       <c r="AD4" s="44"/>
       <c r="AE4" s="4"/>
-      <c r="AF4" s="93" t="s">
+      <c r="AF4" s="97" t="s">
         <v>56</v>
       </c>
-      <c r="AG4" s="94"/>
-      <c r="AH4" s="94"/>
-      <c r="AI4" s="94"/>
-      <c r="AJ4" s="94"/>
-      <c r="AK4" s="94"/>
-      <c r="AL4" s="94"/>
-      <c r="AM4" s="94"/>
-      <c r="AN4" s="95"/>
+      <c r="AG4" s="98"/>
+      <c r="AH4" s="98"/>
+      <c r="AI4" s="98"/>
+      <c r="AJ4" s="98"/>
+      <c r="AK4" s="98"/>
+      <c r="AL4" s="98"/>
+      <c r="AM4" s="98"/>
+      <c r="AN4" s="99"/>
     </row>
     <row r="5" spans="9:40" x14ac:dyDescent="0.3">
       <c r="I5" s="27" t="str">
@@ -5198,32 +4958,32 @@
       <c r="M37" s="25"/>
       <c r="N37" s="25"/>
       <c r="O37" s="25"/>
-      <c r="T37" s="96" t="s">
+      <c r="T37" s="100" t="s">
         <v>87</v>
       </c>
-      <c r="U37" s="97"/>
-      <c r="V37" s="97"/>
-      <c r="W37" s="97"/>
-      <c r="X37" s="97"/>
-      <c r="Y37" s="97"/>
-      <c r="Z37" s="97"/>
-      <c r="AA37" s="97"/>
-      <c r="AB37" s="97"/>
-      <c r="AC37" s="97"/>
-      <c r="AD37" s="98"/>
-      <c r="AF37" s="99" t="s">
+      <c r="U37" s="101"/>
+      <c r="V37" s="101"/>
+      <c r="W37" s="101"/>
+      <c r="X37" s="101"/>
+      <c r="Y37" s="101"/>
+      <c r="Z37" s="101"/>
+      <c r="AA37" s="101"/>
+      <c r="AB37" s="101"/>
+      <c r="AC37" s="101"/>
+      <c r="AD37" s="102"/>
+      <c r="AF37" s="103" t="s">
         <v>87</v>
       </c>
-      <c r="AG37" s="100"/>
-      <c r="AH37" s="100"/>
-      <c r="AI37" s="100"/>
-      <c r="AJ37" s="100"/>
-      <c r="AK37" s="100"/>
-      <c r="AL37" s="100"/>
-      <c r="AM37" s="100"/>
-      <c r="AN37" s="100"/>
-      <c r="AO37" s="100"/>
-      <c r="AP37" s="101"/>
+      <c r="AG37" s="104"/>
+      <c r="AH37" s="104"/>
+      <c r="AI37" s="104"/>
+      <c r="AJ37" s="104"/>
+      <c r="AK37" s="104"/>
+      <c r="AL37" s="104"/>
+      <c r="AM37" s="104"/>
+      <c r="AN37" s="104"/>
+      <c r="AO37" s="104"/>
+      <c r="AP37" s="105"/>
     </row>
     <row r="38" spans="9:42" x14ac:dyDescent="0.3">
       <c r="I38" s="22" t="s">
@@ -5329,40 +5089,40 @@
       <c r="U39" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="V39" s="23" cm="1">
-        <f t="array" aca="1" ref="V39:V46" ca="1">_xlfn._xlws.FILTER(T39:T46, T39:T46=MAX(T39:T46))</f>
-        <v>0</v>
-      </c>
-      <c r="W39" s="23" t="str" cm="1">
-        <f t="array" aca="1" ref="W39:W46" ca="1">_xlfn._xlws.FILTER(ADDRESS(ROW(T39:T46), COLUMN(T39:T46), 4), T39:T46=MAX(T39:T46))</f>
+      <c r="V39" s="23">
+        <f t="array" aca="1" ref="V39" ca="1">_xlfn._xlws.FILTER(T39:T46, T39:T46=MAX(T39:T46))</f>
+        <v>0</v>
+      </c>
+      <c r="W39" s="23" t="str">
+        <f t="array" aca="1" ref="W39" ca="1">_xlfn._xlws.FILTER(ADDRESS(ROW(T39:T46), COLUMN(T39:T46), 4), T39:T46=MAX(T39:T46))</f>
         <v>T39</v>
       </c>
-      <c r="X39" s="23" t="str" cm="1">
-        <f t="array" aca="1" ref="X39:X46" ca="1">_xlfn._xlws.FILTER(U39:U46, T39:T46=MAX(T39:T46))</f>
+      <c r="X39" s="23" t="str">
+        <f t="array" aca="1" ref="X39" ca="1">_xlfn._xlws.FILTER(U39:U46, T39:T46=MAX(T39:T46))</f>
         <v>K6</v>
       </c>
-      <c r="Y39" s="23" t="str" cm="1">
-        <f t="array" aca="1" ref="Y39:Y46" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(X39), _xlfn.LAMBDA(_xlpm.cell_address, INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))-1, COLUMN(INDIRECT(_xlpm.cell_address))-2))))</f>
+      <c r="Y39" s="23" t="str">
+        <f t="array" aca="1" ref="Y39" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(X39), _xlfn.LAMBDA(_xlpm.cell_address, INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))-1, COLUMN(INDIRECT(_xlpm.cell_address))-2))))</f>
         <v>01_Home</v>
       </c>
       <c r="Z39" s="23" t="str">
-        <f ca="1">_xlfn.TEXTJOIN(", ", TRUE,_xlfn.ANCHORARRAY( Y39))</f>
-        <v>01_Home, 02_Testing, 03_About, 04_News, 05_Careers, 06_Contact, 07_Privacy, 08_Game Testing</v>
-      </c>
-      <c r="AA39" s="23" t="str" cm="1">
-        <f t="array" aca="1" ref="AA39:AA46" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(X39), _xlfn.LAMBDA(_xlpm.cell_address, MID(INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))-1, COLUMN(INDIRECT(_xlpm.cell_address))-2)), FIND("_", INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))-1, COLUMN(INDIRECT(_xlpm.cell_address))-2)))+1, 999)))</f>
+        <f t="array" aca="1" ref="Z39" ca="1">_xlfn.TEXTJOIN(", ", TRUE,_xlfn.ANCHORARRAY( Y39))</f>
+        <v>01_Home</v>
+      </c>
+      <c r="AA39" s="23" t="str">
+        <f t="array" aca="1" ref="AA39" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(X39), _xlfn.LAMBDA(_xlpm.cell_address, MID(INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))-1, COLUMN(INDIRECT(_xlpm.cell_address))-2)), FIND("_", INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))-1, COLUMN(INDIRECT(_xlpm.cell_address))-2)))+1, 999)))</f>
         <v>Home</v>
       </c>
       <c r="AB39" s="23" t="str">
-        <f ca="1">_xlfn.TEXTJOIN(", ", TRUE,_xlfn.ANCHORARRAY( AA39))</f>
-        <v>Home, Testing, About, News, Careers, Contact, Privacy, Game Testing</v>
-      </c>
-      <c r="AC39" s="23" t="str" cm="1">
-        <f t="array" aca="1" ref="AC39:AC46" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(X39), _xlfn.LAMBDA(_xlpm.cell_address, INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address)), COLUMN(INDIRECT(_xlpm.cell_address))-1))))</f>
+        <f t="array" aca="1" ref="AB39" ca="1">_xlfn.TEXTJOIN(", ", TRUE,_xlfn.ANCHORARRAY( AA39))</f>
+        <v>Home</v>
+      </c>
+      <c r="AC39" s="23" t="str">
+        <f t="array" aca="1" ref="AC39" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(X39), _xlfn.LAMBDA(_xlpm.cell_address, INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address)), COLUMN(INDIRECT(_xlpm.cell_address))-1))))</f>
         <v>Desktop</v>
       </c>
-      <c r="AD39" s="46" t="str" cm="1">
-        <f t="array" aca="1" ref="AD39:AD46" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(X39), _xlfn.LAMBDA(_xlpm.cell_address, INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))+1, COLUMN(INDIRECT(_xlpm.cell_address))-1))))</f>
+      <c r="AD39" s="46" t="str">
+        <f t="array" aca="1" ref="AD39" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(X39), _xlfn.LAMBDA(_xlpm.cell_address, INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))+1, COLUMN(INDIRECT(_xlpm.cell_address))-1))))</f>
         <v>with and without cache</v>
       </c>
       <c r="AF39" s="54">
@@ -5372,40 +5132,40 @@
       <c r="AG39" t="s">
         <v>69</v>
       </c>
-      <c r="AH39" cm="1">
-        <f t="array" aca="1" ref="AH39:AH45" ca="1">_xlfn._xlws.FILTER(AF39:AF46, AF39:AF46=MIN(AF39:AF46))</f>
-        <v>0</v>
-      </c>
-      <c r="AI39" t="str" cm="1">
-        <f t="array" aca="1" ref="AI39:AI45" ca="1">_xlfn._xlws.FILTER(ADDRESS(ROW(AF39:AF46), COLUMN(AF39:AF46), 4), AF39:AF46=MIN(AF39:AF46))</f>
+      <c r="AH39">
+        <f t="array" aca="1" ref="AH39" ca="1">_xlfn._xlws.FILTER(AF39:AF46, AF39:AF46=MIN(AF39:AF46))</f>
+        <v>0</v>
+      </c>
+      <c r="AI39" t="str">
+        <f t="array" aca="1" ref="AI39" ca="1">_xlfn._xlws.FILTER(ADDRESS(ROW(AF39:AF46), COLUMN(AF39:AF46), 4), AF39:AF46=MIN(AF39:AF46))</f>
         <v>AF39</v>
       </c>
-      <c r="AJ39" t="str" cm="1">
-        <f t="array" aca="1" ref="AJ39:AJ45" ca="1">_xlfn._xlws.FILTER(AG39:AG46, AF39:AF46=MIN(AF39:AF46))</f>
+      <c r="AJ39" t="str">
+        <f t="array" aca="1" ref="AJ39" ca="1">_xlfn._xlws.FILTER(AG39:AG46, AF39:AF46=MIN(AF39:AF46))</f>
         <v>N6</v>
       </c>
-      <c r="AK39" t="str" cm="1">
-        <f t="array" aca="1" ref="AK39:AK45" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(AJ39), _xlfn.LAMBDA(_xlpm.cell_address, INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))-1, COLUMN(INDIRECT(_xlpm.cell_address))-5))))</f>
+      <c r="AK39" t="str">
+        <f t="array" aca="1" ref="AK39" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(AJ39), _xlfn.LAMBDA(_xlpm.cell_address, INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))-1, COLUMN(INDIRECT(_xlpm.cell_address))-5))))</f>
         <v>01_Home</v>
       </c>
       <c r="AL39" t="str">
-        <f ca="1">_xlfn.TEXTJOIN(", ", TRUE, AK39, AK40, AK41, AK42, AK43, AK44, AK45, AK46)</f>
-        <v>01_Home, 02_Testing, 03_About, 04_News, 05_Careers, 07_Privacy, 08_Game Testing</v>
-      </c>
-      <c r="AM39" t="str" cm="1">
-        <f t="array" aca="1" ref="AM39:AM45" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(AJ39), _xlfn.LAMBDA(_xlpm.cell_address, MID(INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))-1, COLUMN(INDIRECT(_xlpm.cell_address))-5)), FIND("_", INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))-1, COLUMN(INDIRECT(_xlpm.cell_address))-5)))+1, 999)))</f>
+        <f t="array" aca="1" ref="AL39" ca="1">_xlfn.TEXTJOIN(", ", TRUE,_xlfn.ANCHORARRAY( AK39))</f>
+        <v>01_Home</v>
+      </c>
+      <c r="AM39" t="str">
+        <f t="array" aca="1" ref="AM39" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(AJ39), _xlfn.LAMBDA(_xlpm.cell_address, MID(INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))-1, COLUMN(INDIRECT(_xlpm.cell_address))-5)), FIND("_", INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))-1, COLUMN(INDIRECT(_xlpm.cell_address))-5)))+1, 999)))</f>
         <v>Home</v>
       </c>
       <c r="AN39" t="str">
-        <f ca="1">_xlfn.TEXTJOIN(", ", TRUE, AM39, AM40, AM41, AM42, AM43, AM44, AM45, AM46)</f>
-        <v>Home, Testing, About, News, Careers, Privacy, Game Testing</v>
-      </c>
-      <c r="AO39" s="23" t="str" cm="1">
-        <f t="array" aca="1" ref="AO39:AO45" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(AJ39), _xlfn.LAMBDA(_xlpm.cell_address, INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address)), COLUMN(INDIRECT(_xlpm.cell_address))-1))))</f>
+        <f t="array" aca="1" ref="AN39" ca="1">_xlfn.TEXTJOIN(", ", TRUE,_xlfn.ANCHORARRAY( AM39))</f>
+        <v>Home</v>
+      </c>
+      <c r="AO39" s="23" t="str">
+        <f t="array" aca="1" ref="AO39" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(AJ39), _xlfn.LAMBDA(_xlpm.cell_address, INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address)), COLUMN(INDIRECT(_xlpm.cell_address))-1))))</f>
         <v>Desktop</v>
       </c>
-      <c r="AP39" s="46" t="str" cm="1">
-        <f t="array" aca="1" ref="AP39:AP45" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(AJ39), _xlfn.LAMBDA(_xlpm.cell_address, INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))+1, COLUMN(INDIRECT(_xlpm.cell_address))-1))))</f>
+      <c r="AP39" s="46" t="str">
+        <f t="array" aca="1" ref="AP39" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(AJ39), _xlfn.LAMBDA(_xlpm.cell_address, INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))+1, COLUMN(INDIRECT(_xlpm.cell_address))-1))))</f>
         <v>with and without cache</v>
       </c>
     </row>
@@ -5432,36 +5192,15 @@
       <c r="U40" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="V40" s="23">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-      <c r="W40" s="23" t="str">
-        <f ca="1"/>
-        <v>T40</v>
-      </c>
-      <c r="X40" s="23" t="str">
-        <f ca="1"/>
-        <v>K10</v>
-      </c>
-      <c r="Y40" s="23" t="str">
-        <f ca="1"/>
-        <v>02_Testing</v>
-      </c>
+      <c r="V40" s="23"/>
+      <c r="W40" s="23"/>
+      <c r="X40" s="23"/>
+      <c r="Y40" s="23"/>
       <c r="Z40" s="23"/>
-      <c r="AA40" s="23" t="str">
-        <f ca="1"/>
-        <v>Testing</v>
-      </c>
+      <c r="AA40" s="23"/>
       <c r="AB40" s="23"/>
-      <c r="AC40" s="23" t="str">
-        <f ca="1"/>
-        <v>Desktop</v>
-      </c>
-      <c r="AD40" s="46" t="str">
-        <f ca="1"/>
-        <v>with and without cache</v>
-      </c>
+      <c r="AC40" s="23"/>
+      <c r="AD40" s="46"/>
       <c r="AF40" s="54">
         <f ca="1">IF(M11="with and without cache", N10, FALSE)</f>
         <v>0</v>
@@ -5469,34 +5208,7 @@
       <c r="AG40" t="s">
         <v>70</v>
       </c>
-      <c r="AH40">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-      <c r="AI40" t="str">
-        <f ca="1"/>
-        <v>AF40</v>
-      </c>
-      <c r="AJ40" t="str">
-        <f ca="1"/>
-        <v>N10</v>
-      </c>
-      <c r="AK40" t="str">
-        <f ca="1"/>
-        <v>02_Testing</v>
-      </c>
-      <c r="AM40" t="str">
-        <f ca="1"/>
-        <v>Testing</v>
-      </c>
-      <c r="AO40" t="str">
-        <f ca="1"/>
-        <v>Desktop</v>
-      </c>
-      <c r="AP40" s="53" t="str">
-        <f ca="1"/>
-        <v>with and without cache</v>
-      </c>
+      <c r="AP40" s="53"/>
     </row>
     <row r="41" spans="9:42" x14ac:dyDescent="0.3">
       <c r="I41" s="22" t="s">
@@ -5521,36 +5233,15 @@
       <c r="U41" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="V41" s="23">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-      <c r="W41" s="23" t="str">
-        <f ca="1"/>
-        <v>T41</v>
-      </c>
-      <c r="X41" s="23" t="str">
-        <f ca="1"/>
-        <v>K14</v>
-      </c>
-      <c r="Y41" s="23" t="str">
-        <f ca="1"/>
-        <v>03_About</v>
-      </c>
+      <c r="V41" s="23"/>
+      <c r="W41" s="23"/>
+      <c r="X41" s="23"/>
+      <c r="Y41" s="23"/>
       <c r="Z41" s="23"/>
-      <c r="AA41" s="23" t="str">
-        <f ca="1"/>
-        <v>About</v>
-      </c>
+      <c r="AA41" s="23"/>
       <c r="AB41" s="23"/>
-      <c r="AC41" s="23" t="str">
-        <f ca="1"/>
-        <v>Desktop</v>
-      </c>
-      <c r="AD41" s="46" t="str">
-        <f ca="1"/>
-        <v>with and without cache</v>
-      </c>
+      <c r="AC41" s="23"/>
+      <c r="AD41" s="46"/>
       <c r="AF41" s="54">
         <f ca="1">IF(M15="with and without cache", N14, FALSE)</f>
         <v>0</v>
@@ -5558,34 +5249,7 @@
       <c r="AG41" s="55" t="s">
         <v>71</v>
       </c>
-      <c r="AH41">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-      <c r="AI41" t="str">
-        <f ca="1"/>
-        <v>AF41</v>
-      </c>
-      <c r="AJ41" t="str">
-        <f ca="1"/>
-        <v>N14</v>
-      </c>
-      <c r="AK41" t="str">
-        <f ca="1"/>
-        <v>03_About</v>
-      </c>
-      <c r="AM41" t="str">
-        <f ca="1"/>
-        <v>About</v>
-      </c>
-      <c r="AO41" t="str">
-        <f ca="1"/>
-        <v>Desktop</v>
-      </c>
-      <c r="AP41" s="53" t="str">
-        <f ca="1"/>
-        <v>with and without cache</v>
-      </c>
+      <c r="AP41" s="53"/>
     </row>
     <row r="42" spans="9:42" x14ac:dyDescent="0.3">
       <c r="I42" s="22" t="s">
@@ -5616,36 +5280,15 @@
       <c r="U42" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="V42" s="23">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-      <c r="W42" s="23" t="str">
-        <f ca="1"/>
-        <v>T42</v>
-      </c>
-      <c r="X42" s="23" t="str">
-        <f ca="1"/>
-        <v>K18</v>
-      </c>
-      <c r="Y42" s="23" t="str">
-        <f ca="1"/>
-        <v>04_News</v>
-      </c>
+      <c r="V42" s="23"/>
+      <c r="W42" s="23"/>
+      <c r="X42" s="23"/>
+      <c r="Y42" s="23"/>
       <c r="Z42" s="23"/>
-      <c r="AA42" s="23" t="str">
-        <f ca="1"/>
-        <v>News</v>
-      </c>
+      <c r="AA42" s="23"/>
       <c r="AB42" s="23"/>
-      <c r="AC42" s="23" t="str">
-        <f ca="1"/>
-        <v>Desktop</v>
-      </c>
-      <c r="AD42" s="46" t="str">
-        <f ca="1"/>
-        <v>with and without cache</v>
-      </c>
+      <c r="AC42" s="23"/>
+      <c r="AD42" s="46"/>
       <c r="AF42" s="54">
         <f ca="1">IF(M19="with and without cache", N18, FALSE)</f>
         <v>0</v>
@@ -5653,34 +5296,7 @@
       <c r="AG42" t="s">
         <v>72</v>
       </c>
-      <c r="AH42">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-      <c r="AI42" t="str">
-        <f ca="1"/>
-        <v>AF42</v>
-      </c>
-      <c r="AJ42" t="str">
-        <f ca="1"/>
-        <v>N18</v>
-      </c>
-      <c r="AK42" t="str">
-        <f ca="1"/>
-        <v>04_News</v>
-      </c>
-      <c r="AM42" t="str">
-        <f ca="1"/>
-        <v>News</v>
-      </c>
-      <c r="AO42" t="str">
-        <f ca="1"/>
-        <v>Desktop</v>
-      </c>
-      <c r="AP42" s="53" t="str">
-        <f ca="1"/>
-        <v>with and without cache</v>
-      </c>
+      <c r="AP42" s="53"/>
     </row>
     <row r="43" spans="9:42" x14ac:dyDescent="0.3">
       <c r="I43" s="22" t="s">
@@ -5711,36 +5327,15 @@
       <c r="U43" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="V43" s="23">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-      <c r="W43" s="23" t="str">
-        <f ca="1"/>
-        <v>T43</v>
-      </c>
-      <c r="X43" s="23" t="str">
-        <f ca="1"/>
-        <v>K22</v>
-      </c>
-      <c r="Y43" s="23" t="str">
-        <f ca="1"/>
-        <v>05_Careers</v>
-      </c>
+      <c r="V43" s="23"/>
+      <c r="W43" s="23"/>
+      <c r="X43" s="23"/>
+      <c r="Y43" s="23"/>
       <c r="Z43" s="23"/>
-      <c r="AA43" s="23" t="str">
-        <f ca="1"/>
-        <v>Careers</v>
-      </c>
+      <c r="AA43" s="23"/>
       <c r="AB43" s="23"/>
-      <c r="AC43" s="23" t="str">
-        <f ca="1"/>
-        <v>Desktop</v>
-      </c>
-      <c r="AD43" s="46" t="str">
-        <f ca="1"/>
-        <v>with and without cache</v>
-      </c>
+      <c r="AC43" s="23"/>
+      <c r="AD43" s="46"/>
       <c r="AF43" s="54">
         <f ca="1">IF(M23="with and without cache", N22, FALSE)</f>
         <v>0</v>
@@ -5748,34 +5343,7 @@
       <c r="AG43" t="s">
         <v>73</v>
       </c>
-      <c r="AH43">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-      <c r="AI43" t="str">
-        <f ca="1"/>
-        <v>AF43</v>
-      </c>
-      <c r="AJ43" t="str">
-        <f ca="1"/>
-        <v>N22</v>
-      </c>
-      <c r="AK43" t="str">
-        <f ca="1"/>
-        <v>05_Careers</v>
-      </c>
-      <c r="AM43" t="str">
-        <f ca="1"/>
-        <v>Careers</v>
-      </c>
-      <c r="AO43" t="str">
-        <f ca="1"/>
-        <v>Desktop</v>
-      </c>
-      <c r="AP43" s="53" t="str">
-        <f ca="1"/>
-        <v>with and without cache</v>
-      </c>
+      <c r="AP43" s="53"/>
     </row>
     <row r="44" spans="9:42" x14ac:dyDescent="0.3">
       <c r="I44" s="22" t="s">
@@ -5814,36 +5382,15 @@
       <c r="U44" s="23" t="s">
         <v>66</v>
       </c>
-      <c r="V44" s="23">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-      <c r="W44" s="23" t="str">
-        <f ca="1"/>
-        <v>T44</v>
-      </c>
-      <c r="X44" s="23" t="str">
-        <f ca="1"/>
-        <v>K26</v>
-      </c>
-      <c r="Y44" s="23" t="str">
-        <f ca="1"/>
-        <v>06_Contact</v>
-      </c>
+      <c r="V44" s="23"/>
+      <c r="W44" s="23"/>
+      <c r="X44" s="23"/>
+      <c r="Y44" s="23"/>
       <c r="Z44" s="23"/>
-      <c r="AA44" s="23" t="str">
-        <f ca="1"/>
-        <v>Contact</v>
-      </c>
+      <c r="AA44" s="23"/>
       <c r="AB44" s="23"/>
-      <c r="AC44" s="23" t="str">
-        <f ca="1"/>
-        <v>Desktop</v>
-      </c>
-      <c r="AD44" s="46" t="str">
-        <f ca="1"/>
-        <v>with and without cache</v>
-      </c>
+      <c r="AC44" s="23"/>
+      <c r="AD44" s="46"/>
       <c r="AF44" s="54" t="b">
         <f ca="1">IF(M26="with and without cache", N26, FALSE)</f>
         <v>0</v>
@@ -5851,34 +5398,7 @@
       <c r="AG44" t="s">
         <v>74</v>
       </c>
-      <c r="AH44">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-      <c r="AI44" t="str">
-        <f ca="1"/>
-        <v>AF45</v>
-      </c>
-      <c r="AJ44" t="str">
-        <f ca="1"/>
-        <v>N30</v>
-      </c>
-      <c r="AK44" t="str">
-        <f ca="1"/>
-        <v>07_Privacy</v>
-      </c>
-      <c r="AM44" t="str">
-        <f ca="1"/>
-        <v>Privacy</v>
-      </c>
-      <c r="AO44" t="str">
-        <f ca="1"/>
-        <v>Desktop</v>
-      </c>
-      <c r="AP44" s="53" t="str">
-        <f ca="1"/>
-        <v>with and without cache</v>
-      </c>
+      <c r="AP44" s="53"/>
     </row>
     <row r="45" spans="9:42" x14ac:dyDescent="0.3">
       <c r="I45" s="22" t="s">
@@ -5911,36 +5431,15 @@
       <c r="U45" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="V45" s="23">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-      <c r="W45" s="23" t="str">
-        <f ca="1"/>
-        <v>T45</v>
-      </c>
-      <c r="X45" s="23" t="str">
-        <f ca="1"/>
-        <v>K30</v>
-      </c>
-      <c r="Y45" s="23" t="str">
-        <f ca="1"/>
-        <v>07_Privacy</v>
-      </c>
+      <c r="V45" s="23"/>
+      <c r="W45" s="23"/>
+      <c r="X45" s="23"/>
+      <c r="Y45" s="23"/>
       <c r="Z45" s="23"/>
-      <c r="AA45" s="23" t="str">
-        <f ca="1"/>
-        <v>Privacy</v>
-      </c>
+      <c r="AA45" s="23"/>
       <c r="AB45" s="23"/>
-      <c r="AC45" s="23" t="str">
-        <f ca="1"/>
-        <v>Desktop</v>
-      </c>
-      <c r="AD45" s="46" t="str">
-        <f ca="1"/>
-        <v>with and without cache</v>
-      </c>
+      <c r="AC45" s="23"/>
+      <c r="AD45" s="46"/>
       <c r="AF45" s="54">
         <f ca="1">IF(M31="with and without cache", N30, FALSE)</f>
         <v>0</v>
@@ -5948,34 +5447,7 @@
       <c r="AG45" t="s">
         <v>75</v>
       </c>
-      <c r="AH45">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-      <c r="AI45" t="str">
-        <f ca="1"/>
-        <v>AF46</v>
-      </c>
-      <c r="AJ45" t="str">
-        <f ca="1"/>
-        <v>N34</v>
-      </c>
-      <c r="AK45" t="str">
-        <f ca="1"/>
-        <v>08_Game Testing</v>
-      </c>
-      <c r="AM45" t="str">
-        <f ca="1"/>
-        <v>Game Testing</v>
-      </c>
-      <c r="AO45" t="str">
-        <f ca="1"/>
-        <v>Desktop</v>
-      </c>
-      <c r="AP45" s="53" t="str">
-        <f ca="1"/>
-        <v>with and without cache</v>
-      </c>
+      <c r="AP45" s="53"/>
     </row>
     <row r="46" spans="9:42" x14ac:dyDescent="0.3">
       <c r="I46" s="22" t="s">
@@ -5996,36 +5468,15 @@
       <c r="U46" s="48" t="s">
         <v>68</v>
       </c>
-      <c r="V46" s="48">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-      <c r="W46" s="48" t="str">
-        <f ca="1"/>
-        <v>T46</v>
-      </c>
-      <c r="X46" s="48" t="str">
-        <f ca="1"/>
-        <v>K34</v>
-      </c>
-      <c r="Y46" s="48" t="str">
-        <f ca="1"/>
-        <v>08_Game Testing</v>
-      </c>
+      <c r="V46" s="48"/>
+      <c r="W46" s="48"/>
+      <c r="X46" s="48"/>
+      <c r="Y46" s="48"/>
       <c r="Z46" s="48"/>
-      <c r="AA46" s="48" t="str">
-        <f ca="1"/>
-        <v>Game Testing</v>
-      </c>
+      <c r="AA46" s="48"/>
       <c r="AB46" s="48"/>
-      <c r="AC46" s="48" t="str">
-        <f ca="1"/>
-        <v>Desktop</v>
-      </c>
-      <c r="AD46" s="49" t="str">
-        <f ca="1"/>
-        <v>with and without cache</v>
-      </c>
+      <c r="AC46" s="48"/>
+      <c r="AD46" s="49"/>
       <c r="AF46" s="56">
         <f ca="1">IF(M35="with and without cache", N34, FALSE)</f>
         <v>0</v>
@@ -6054,37 +5505,37 @@
       </c>
       <c r="AH47">
         <f ca="1">COUNT(AH39:AH46)</f>
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48" spans="9:42" x14ac:dyDescent="0.3">
       <c r="M48" s="25"/>
-      <c r="T48" s="96" t="s">
+      <c r="T48" s="100" t="s">
         <v>88</v>
       </c>
-      <c r="U48" s="97"/>
-      <c r="V48" s="97"/>
-      <c r="W48" s="97"/>
-      <c r="X48" s="97"/>
-      <c r="Y48" s="97"/>
-      <c r="Z48" s="97"/>
-      <c r="AA48" s="97"/>
-      <c r="AB48" s="97"/>
-      <c r="AC48" s="97"/>
-      <c r="AD48" s="98"/>
-      <c r="AF48" s="99" t="s">
+      <c r="U48" s="101"/>
+      <c r="V48" s="101"/>
+      <c r="W48" s="101"/>
+      <c r="X48" s="101"/>
+      <c r="Y48" s="101"/>
+      <c r="Z48" s="101"/>
+      <c r="AA48" s="101"/>
+      <c r="AB48" s="101"/>
+      <c r="AC48" s="101"/>
+      <c r="AD48" s="102"/>
+      <c r="AF48" s="103" t="s">
         <v>88</v>
       </c>
-      <c r="AG48" s="100"/>
-      <c r="AH48" s="100"/>
-      <c r="AI48" s="100"/>
-      <c r="AJ48" s="100"/>
-      <c r="AK48" s="100"/>
-      <c r="AL48" s="100"/>
-      <c r="AM48" s="100"/>
-      <c r="AN48" s="100"/>
-      <c r="AO48" s="100"/>
-      <c r="AP48" s="101"/>
+      <c r="AG48" s="104"/>
+      <c r="AH48" s="104"/>
+      <c r="AI48" s="104"/>
+      <c r="AJ48" s="104"/>
+      <c r="AK48" s="104"/>
+      <c r="AL48" s="104"/>
+      <c r="AM48" s="104"/>
+      <c r="AN48" s="104"/>
+      <c r="AO48" s="104"/>
+      <c r="AP48" s="105"/>
     </row>
     <row r="49" spans="13:42" x14ac:dyDescent="0.3">
       <c r="M49"/>
@@ -6163,39 +5614,39 @@
       <c r="U50" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="V50" s="25" cm="1">
+      <c r="V50" s="25">
         <f t="array" aca="1" ref="V50" ca="1">_xlfn._xlws.FILTER(T50:T57, T50:T57=MAX(T50:T57))</f>
         <v>-1</v>
       </c>
-      <c r="W50" s="23" t="str" cm="1">
+      <c r="W50" s="23" t="str">
         <f t="array" aca="1" ref="W50" ca="1">_xlfn._xlws.FILTER(ADDRESS(ROW(T50:T57), COLUMN(T50:T57), 4), T50:T57=MAX(T50:T57))</f>
         <v>T50</v>
       </c>
-      <c r="X50" s="23" t="str" cm="1">
+      <c r="X50" s="23" t="str">
         <f t="array" aca="1" ref="X50" ca="1">_xlfn._xlws.FILTER(U50:U57, T50:T57=MAX(T50:T57))</f>
         <v>K6</v>
       </c>
-      <c r="Y50" s="23" t="str" cm="1">
+      <c r="Y50" s="23" t="str">
         <f t="array" aca="1" ref="Y50" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(X50), _xlfn.LAMBDA(_xlpm.cell_address, INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))-1, COLUMN(INDIRECT(_xlpm.cell_address))-2))))</f>
         <v>01_Home</v>
       </c>
       <c r="Z50" s="23" t="str">
-        <f ca="1">_xlfn.TEXTJOIN(", ", TRUE,_xlfn.ANCHORARRAY( Y50))</f>
+        <f t="array" aca="1" ref="Z50" ca="1">_xlfn.TEXTJOIN(", ", TRUE,_xlfn.ANCHORARRAY( Y50))</f>
         <v>01_Home</v>
       </c>
-      <c r="AA50" s="23" t="str" cm="1">
+      <c r="AA50" s="23" t="str">
         <f t="array" aca="1" ref="AA50" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(X50), _xlfn.LAMBDA(_xlpm.cell_address, MID(INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))-1, COLUMN(INDIRECT(_xlpm.cell_address))-2)), FIND("_", INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))-1, COLUMN(INDIRECT(_xlpm.cell_address))-2)))+1, 999)))</f>
         <v>Home</v>
       </c>
       <c r="AB50" s="23" t="str">
-        <f ca="1">_xlfn.TEXTJOIN(", ", TRUE,_xlfn.ANCHORARRAY( AA50))</f>
+        <f t="array" aca="1" ref="AB50" ca="1">_xlfn.TEXTJOIN(", ", TRUE,_xlfn.ANCHORARRAY( AA50))</f>
         <v>Home</v>
       </c>
-      <c r="AC50" s="23" t="str" cm="1">
+      <c r="AC50" s="23" t="str">
         <f t="array" aca="1" ref="AC50" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(X50), _xlfn.LAMBDA(_xlpm.cell_address, INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address)), COLUMN(INDIRECT(_xlpm.cell_address))-1))))</f>
         <v>Desktop</v>
       </c>
-      <c r="AD50" s="46" t="str" cm="1">
+      <c r="AD50" s="46" t="str">
         <f t="array" aca="1" ref="AD50" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(X50), _xlfn.LAMBDA(_xlpm.cell_address, INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))+1, COLUMN(INDIRECT(_xlpm.cell_address))-1))))</f>
         <v>with and without cache</v>
       </c>
@@ -6206,39 +5657,39 @@
       <c r="AG50" t="s">
         <v>69</v>
       </c>
-      <c r="AH50" s="25" cm="1">
+      <c r="AH50" s="25">
         <f t="array" aca="1" ref="AH50" ca="1">_xlfn._xlws.FILTER(AF50:AF57, AF50:AF57=MIN(AF50:AF57))</f>
         <v>99999</v>
       </c>
-      <c r="AI50" s="23" t="str" cm="1">
+      <c r="AI50" s="23" t="str">
         <f t="array" aca="1" ref="AI50" ca="1">_xlfn._xlws.FILTER(ADDRESS(ROW(AF50:AF57), COLUMN(AF50:AF57), 4), AF50:AF57=MIN(AF50:AF57))</f>
         <v>AF50</v>
       </c>
-      <c r="AJ50" s="23" t="str" cm="1">
+      <c r="AJ50" s="23" t="str">
         <f t="array" aca="1" ref="AJ50" ca="1">_xlfn._xlws.FILTER(AG50:AG57, AF50:AF57=MIN(AF50:AF57))</f>
         <v>N6</v>
       </c>
-      <c r="AK50" s="23" t="str" cm="1">
+      <c r="AK50" s="23" t="str">
         <f t="array" aca="1" ref="AK50" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(AJ50), _xlfn.LAMBDA(_xlpm.cell_address, INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))-1, COLUMN(INDIRECT(_xlpm.cell_address))-5))))</f>
         <v>01_Home</v>
       </c>
       <c r="AL50" s="23" t="str">
-        <f ca="1">_xlfn.TEXTJOIN(", ", TRUE,_xlfn.ANCHORARRAY( AK50))</f>
+        <f t="array" aca="1" ref="AL50" ca="1">_xlfn.TEXTJOIN(", ", TRUE,_xlfn.ANCHORARRAY( AK50))</f>
         <v>01_Home</v>
       </c>
-      <c r="AM50" s="23" t="str" cm="1">
+      <c r="AM50" s="23" t="str">
         <f t="array" aca="1" ref="AM50" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(AJ50), _xlfn.LAMBDA(_xlpm.cell_address, MID(INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))-1, COLUMN(INDIRECT(_xlpm.cell_address))-5)), FIND("_", INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))-1, COLUMN(INDIRECT(_xlpm.cell_address))-5)))+1, 999)))</f>
         <v>Home</v>
       </c>
       <c r="AN50" s="23" t="str">
-        <f ca="1">_xlfn.TEXTJOIN(", ", TRUE,_xlfn.ANCHORARRAY( AM50))</f>
+        <f t="array" aca="1" ref="AN50" ca="1">_xlfn.TEXTJOIN(", ", TRUE,_xlfn.ANCHORARRAY( AM50))</f>
         <v>Home</v>
       </c>
-      <c r="AO50" s="23" t="str" cm="1">
+      <c r="AO50" s="23" t="str">
         <f t="array" aca="1" ref="AO50" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(AJ50), _xlfn.LAMBDA(_xlpm.cell_address, INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address)), COLUMN(INDIRECT(_xlpm.cell_address))-1))))</f>
         <v>Desktop</v>
       </c>
-      <c r="AP50" s="46" t="str" cm="1">
+      <c r="AP50" s="46" t="str">
         <f t="array" aca="1" ref="AP50" ca="1">_xlfn.MAP(_xlfn.ANCHORARRAY(AJ50), _xlfn.LAMBDA(_xlpm.cell_address, INDIRECT(ADDRESS(ROW(INDIRECT(_xlpm.cell_address))+1, COLUMN(INDIRECT(_xlpm.cell_address))-1))))</f>
         <v>with and without cache</v>
       </c>
@@ -6487,7 +5938,7 @@
 IF(Formula_Sheet!V39&gt;=Formula_Sheet!V50,
 _xlfn.TEXTJOIN(", ", TRUE, _xlfn.MAP(_xlfn.ANCHORARRAY(AA39),_xlfn.ANCHORARRAY( AC39),_xlfn.ANCHORARRAY( AD39), _xlfn.LAMBDA(_xlpm.name,_xlpm.device,_xlpm.cache, _xlpm.name &amp; " page for " &amp; _xlpm.device &amp; " devices " &amp; _xlpm.cache))),
 _xlfn.TEXTJOIN(", ", TRUE, _xlfn.MAP(_xlfn.ANCHORARRAY(AA50),_xlfn.ANCHORARRAY( AC50),_xlfn.ANCHORARRAY( AD50), _xlfn.LAMBDA(_xlpm.name,_xlpm.device,_xlpm.cache, _xlpm.name &amp; " page for " &amp; _xlpm.device &amp; " devices " &amp; _xlpm.cache))))</f>
-        <v>The best recorded performance score was in the Home page for Desktop devices with and without cache, Testing page for Desktop devices with and without cache, About page for Desktop devices with and without cache, News page for Desktop devices with and without cache, Careers page for Desktop devices with and without cache, Contact page for Desktop devices with and without cache, Privacy page for Desktop devices with and without cache, Game Testing page for Desktop devices with and without cache</v>
+        <v>The best recorded performance score was in the Home page for Desktop devices with and without cache</v>
       </c>
       <c r="U61" s="59"/>
       <c r="V61" s="59"/>
@@ -6499,7 +5950,7 @@
 IF(Formula_Sheet!AH39&lt;=Formula_Sheet!AH50,
 _xlfn.TEXTJOIN(", ", TRUE, _xlfn.MAP(_xlfn.ANCHORARRAY(AM39),_xlfn.ANCHORARRAY( AO39),_xlfn.ANCHORARRAY( AP39), _xlfn.LAMBDA(_xlpm.name,_xlpm.device,_xlpm.cache, _xlpm.name &amp; " page for " &amp; _xlpm.device &amp; " devices " &amp; _xlpm.cache))),
 _xlfn.TEXTJOIN(", ", TRUE, _xlfn.MAP(_xlfn.ANCHORARRAY(AM50),_xlfn.ANCHORARRAY( AO50),_xlfn.ANCHORARRAY( AP50), _xlfn.LAMBDA(_xlpm.name,_xlpm.device,_xlpm.cache, _xlpm.name &amp; " page for " &amp; _xlpm.device &amp; " devices " &amp; _xlpm.cache))))</f>
-        <v>The worst recorded performance score was in the Home page for Desktop devices with and without cache, Testing page for Desktop devices with and without cache, About page for Desktop devices with and without cache, News page for Desktop devices with and without cache, Careers page for Desktop devices with and without cache, Privacy page for Desktop devices with and without cache, Game Testing page for Desktop devices with and without cache</v>
+        <v>The worst recorded performance score was in the Home page for Desktop devices with and without cache</v>
       </c>
       <c r="AG61" s="60"/>
       <c r="AH61" s="60"/>
@@ -6520,11 +5971,11 @@
     <row r="64" spans="13:42" x14ac:dyDescent="0.3">
       <c r="T64" t="str">
         <f ca="1">"Refer to " &amp;IF(Formula_Sheet!V39&gt;=Formula_Sheet!V50, Formula_Sheet!Z39, Formula_Sheet!Z50)&amp; " tab for the best insight, links for full diagnostic readings and recommendations for improvement."</f>
-        <v>Refer to 01_Home, 02_Testing, 03_About, 04_News, 05_Careers, 06_Contact, 07_Privacy, 08_Game Testing tab for the best insight, links for full diagnostic readings and recommendations for improvement.</v>
+        <v>Refer to 01_Home tab for the best insight, links for full diagnostic readings and recommendations for improvement.</v>
       </c>
       <c r="AF64" t="str">
         <f ca="1">"Refer to " &amp;IF(Formula_Sheet!AH39&lt;=Formula_Sheet!AH50, Formula_Sheet!AL39, Formula_Sheet!AL50)&amp; " tab for the best insight, links for full diagnostic readings and recommendations for improvement."</f>
-        <v>Refer to 01_Home, 02_Testing, 03_About, 04_News, 05_Careers, 07_Privacy, 08_Game Testing tab for the best insight, links for full diagnostic readings and recommendations for improvement.</v>
+        <v>Refer to 01_Home tab for the best insight, links for full diagnostic readings and recommendations for improvement.</v>
       </c>
     </row>
   </sheetData>
@@ -6556,18 +6007,18 @@
   <sheetData>
     <row r="1" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C2" s="81">
+      <c r="C2" s="76">
         <f>Summary!D6</f>
         <v>0</v>
       </c>
-      <c r="D2" s="82"/>
+      <c r="D2" s="77"/>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B3" s="83" t="str">
+      <c r="B3" s="78" t="str">
         <f>Summary!B7</f>
         <v>01_Home</v>
       </c>
-      <c r="C3" s="86" t="s">
+      <c r="C3" s="81" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="18" t="s">
@@ -6576,16 +6027,16 @@
       <c r="E3" s="17"/>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B4" s="84"/>
-      <c r="C4" s="87"/>
+      <c r="B4" s="79"/>
+      <c r="C4" s="82"/>
       <c r="D4" s="19" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="17"/>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B5" s="84"/>
-      <c r="C5" s="87" t="s">
+      <c r="B5" s="79"/>
+      <c r="C5" s="82" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="19" t="s">
@@ -6594,8 +6045,8 @@
       <c r="E5" s="17"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B6" s="85"/>
-      <c r="C6" s="88"/>
+      <c r="B6" s="80"/>
+      <c r="C6" s="83"/>
       <c r="D6" s="20" t="s">
         <v>4</v>
       </c>
@@ -6615,26 +6066,26 @@
       <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="76">
+      <c r="C9" s="84">
         <f>E5</f>
         <v>0</v>
       </c>
-      <c r="D9" s="77"/>
-      <c r="E9" s="78"/>
+      <c r="D9" s="85"/>
+      <c r="E9" s="86"/>
     </row>
     <row r="10" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="72"/>
-      <c r="D10" s="73"/>
+      <c r="C10" s="87"/>
+      <c r="D10" s="88"/>
     </row>
     <row r="11" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="74"/>
-      <c r="D11" s="75"/>
+      <c r="C11" s="89"/>
+      <c r="D11" s="90"/>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C12" s="16"/>
@@ -6665,41 +6116,41 @@
       <c r="B25" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="76">
+      <c r="C25" s="84">
         <f>E5</f>
         <v>0</v>
       </c>
-      <c r="D25" s="77"/>
-      <c r="E25" s="78"/>
+      <c r="D25" s="85"/>
+      <c r="E25" s="86"/>
     </row>
     <row r="26" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="72"/>
-      <c r="D26" s="79"/>
-      <c r="E26" s="73"/>
+      <c r="C26" s="87"/>
+      <c r="D26" s="91"/>
+      <c r="E26" s="88"/>
     </row>
     <row r="27" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="74"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="75"/>
+      <c r="C27" s="89"/>
+      <c r="D27" s="92"/>
+      <c r="E27" s="90"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="C27:E27"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B3:B6"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="C5:C6"/>
     <mergeCell ref="C9:E9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="C26:E26"/>
-    <mergeCell ref="C27:E27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6721,18 +6172,18 @@
   <sheetData>
     <row r="1" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C2" s="81">
+      <c r="C2" s="76">
         <f>Summary!D10</f>
         <v>0</v>
       </c>
-      <c r="D2" s="82"/>
+      <c r="D2" s="77"/>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B3" s="83" t="str">
+      <c r="B3" s="78" t="str">
         <f>Summary!B11</f>
         <v>02_Testing</v>
       </c>
-      <c r="C3" s="86" t="s">
+      <c r="C3" s="81" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="18" t="s">
@@ -6741,16 +6192,16 @@
       <c r="E3" s="17"/>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B4" s="84"/>
-      <c r="C4" s="87"/>
+      <c r="B4" s="79"/>
+      <c r="C4" s="82"/>
       <c r="D4" s="19" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="17"/>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B5" s="84"/>
-      <c r="C5" s="87" t="s">
+      <c r="B5" s="79"/>
+      <c r="C5" s="82" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="19" t="s">
@@ -6759,8 +6210,8 @@
       <c r="E5" s="17"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B6" s="85"/>
-      <c r="C6" s="88"/>
+      <c r="B6" s="80"/>
+      <c r="C6" s="83"/>
       <c r="D6" s="20" t="s">
         <v>4</v>
       </c>
@@ -6780,27 +6231,27 @@
       <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="76">
+      <c r="C9" s="84">
         <f>E5</f>
         <v>0</v>
       </c>
-      <c r="D9" s="77"/>
-      <c r="E9" s="78"/>
+      <c r="D9" s="85"/>
+      <c r="E9" s="86"/>
     </row>
     <row r="10" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="72"/>
-      <c r="D10" s="73"/>
+      <c r="C10" s="87"/>
+      <c r="D10" s="88"/>
       <c r="E10" s="23"/>
     </row>
     <row r="11" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="74"/>
-      <c r="D11" s="75"/>
+      <c r="C11" s="89"/>
+      <c r="D11" s="90"/>
       <c r="E11" s="23"/>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
@@ -6844,28 +6295,28 @@
       <c r="B25" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="76">
+      <c r="C25" s="84">
         <f>E5</f>
         <v>0</v>
       </c>
-      <c r="D25" s="77"/>
-      <c r="E25" s="78"/>
+      <c r="D25" s="85"/>
+      <c r="E25" s="86"/>
     </row>
     <row r="26" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="72"/>
-      <c r="D26" s="79"/>
-      <c r="E26" s="73"/>
+      <c r="C26" s="87"/>
+      <c r="D26" s="91"/>
+      <c r="E26" s="88"/>
     </row>
     <row r="27" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="74"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="75"/>
+      <c r="C27" s="89"/>
+      <c r="D27" s="92"/>
+      <c r="E27" s="90"/>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C30" s="21"/>
@@ -6903,18 +6354,18 @@
   <sheetData>
     <row r="1" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C2" s="81">
+      <c r="C2" s="76">
         <f>Summary!D14</f>
         <v>0</v>
       </c>
-      <c r="D2" s="82"/>
+      <c r="D2" s="77"/>
     </row>
     <row r="3" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="83" t="str">
+      <c r="B3" s="78" t="str">
         <f>Summary!B15</f>
         <v>03_About</v>
       </c>
-      <c r="C3" s="86" t="s">
+      <c r="C3" s="81" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="18" t="s">
@@ -6923,16 +6374,16 @@
       <c r="E3" s="17"/>
     </row>
     <row r="4" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="84"/>
-      <c r="C4" s="87"/>
+      <c r="B4" s="79"/>
+      <c r="C4" s="82"/>
       <c r="D4" s="19" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="17"/>
     </row>
     <row r="5" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="84"/>
-      <c r="C5" s="87" t="s">
+      <c r="B5" s="79"/>
+      <c r="C5" s="82" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="19" t="s">
@@ -6941,8 +6392,8 @@
       <c r="E5" s="17"/>
     </row>
     <row r="6" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="85"/>
-      <c r="C6" s="88"/>
+      <c r="B6" s="80"/>
+      <c r="C6" s="83"/>
       <c r="D6" s="20" t="s">
         <v>4</v>
       </c>
@@ -6962,27 +6413,27 @@
       <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="76">
+      <c r="C9" s="84">
         <f>E5</f>
         <v>0</v>
       </c>
-      <c r="D9" s="77"/>
-      <c r="E9" s="78"/>
+      <c r="D9" s="85"/>
+      <c r="E9" s="86"/>
     </row>
     <row r="10" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="72"/>
-      <c r="D10" s="73"/>
+      <c r="C10" s="87"/>
+      <c r="D10" s="88"/>
       <c r="E10" s="23"/>
     </row>
     <row r="11" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="74"/>
-      <c r="D11" s="75"/>
+      <c r="C11" s="89"/>
+      <c r="D11" s="90"/>
       <c r="E11" s="23"/>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
@@ -7014,28 +6465,28 @@
       <c r="B25" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="76">
+      <c r="C25" s="84">
         <f>E5</f>
         <v>0</v>
       </c>
-      <c r="D25" s="77"/>
-      <c r="E25" s="78"/>
+      <c r="D25" s="85"/>
+      <c r="E25" s="86"/>
     </row>
     <row r="26" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="72"/>
-      <c r="D26" s="79"/>
-      <c r="E26" s="73"/>
+      <c r="C26" s="87"/>
+      <c r="D26" s="91"/>
+      <c r="E26" s="88"/>
     </row>
     <row r="27" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="74"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="75"/>
+      <c r="C27" s="89"/>
+      <c r="D27" s="92"/>
+      <c r="E27" s="90"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -7070,18 +6521,18 @@
   <sheetData>
     <row r="1" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C2" s="81">
+      <c r="C2" s="76">
         <f>Summary!D18</f>
         <v>0</v>
       </c>
-      <c r="D2" s="82"/>
+      <c r="D2" s="77"/>
     </row>
     <row r="3" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="83" t="str">
+      <c r="B3" s="78" t="str">
         <f>Summary!B19</f>
         <v>04_News</v>
       </c>
-      <c r="C3" s="86" t="s">
+      <c r="C3" s="81" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="18" t="s">
@@ -7090,16 +6541,16 @@
       <c r="E3" s="17"/>
     </row>
     <row r="4" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="84"/>
-      <c r="C4" s="87"/>
+      <c r="B4" s="79"/>
+      <c r="C4" s="82"/>
       <c r="D4" s="19" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="17"/>
     </row>
     <row r="5" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="84"/>
-      <c r="C5" s="87" t="s">
+      <c r="B5" s="79"/>
+      <c r="C5" s="82" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="19" t="s">
@@ -7108,8 +6559,8 @@
       <c r="E5" s="17"/>
     </row>
     <row r="6" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="85"/>
-      <c r="C6" s="88"/>
+      <c r="B6" s="80"/>
+      <c r="C6" s="83"/>
       <c r="D6" s="20" t="s">
         <v>4</v>
       </c>
@@ -7129,27 +6580,27 @@
       <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="76">
+      <c r="C9" s="84">
         <f>E5</f>
         <v>0</v>
       </c>
-      <c r="D9" s="77"/>
-      <c r="E9" s="78"/>
+      <c r="D9" s="85"/>
+      <c r="E9" s="86"/>
     </row>
     <row r="10" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="72"/>
-      <c r="D10" s="73"/>
+      <c r="C10" s="87"/>
+      <c r="D10" s="88"/>
       <c r="E10" s="23"/>
     </row>
     <row r="11" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="74"/>
-      <c r="D11" s="75"/>
+      <c r="C11" s="89"/>
+      <c r="D11" s="90"/>
       <c r="E11" s="23"/>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
@@ -7193,28 +6644,28 @@
       <c r="B25" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="76">
+      <c r="C25" s="84">
         <f>E5</f>
         <v>0</v>
       </c>
-      <c r="D25" s="77"/>
-      <c r="E25" s="78"/>
+      <c r="D25" s="85"/>
+      <c r="E25" s="86"/>
     </row>
     <row r="26" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="72"/>
-      <c r="D26" s="79"/>
-      <c r="E26" s="73"/>
+      <c r="C26" s="87"/>
+      <c r="D26" s="91"/>
+      <c r="E26" s="88"/>
     </row>
     <row r="27" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="74"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="75"/>
+      <c r="C27" s="89"/>
+      <c r="D27" s="92"/>
+      <c r="E27" s="90"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -7249,18 +6700,18 @@
   <sheetData>
     <row r="1" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C2" s="81">
+      <c r="C2" s="76">
         <f>Summary!D22</f>
         <v>0</v>
       </c>
-      <c r="D2" s="82"/>
+      <c r="D2" s="77"/>
     </row>
     <row r="3" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="83" t="str">
+      <c r="B3" s="78" t="str">
         <f>Summary!B23</f>
         <v>05_Careers</v>
       </c>
-      <c r="C3" s="86" t="s">
+      <c r="C3" s="81" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="18" t="s">
@@ -7269,16 +6720,16 @@
       <c r="E3" s="17"/>
     </row>
     <row r="4" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="84"/>
-      <c r="C4" s="87"/>
+      <c r="B4" s="79"/>
+      <c r="C4" s="82"/>
       <c r="D4" s="19" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="17"/>
     </row>
     <row r="5" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="84"/>
-      <c r="C5" s="87" t="s">
+      <c r="B5" s="79"/>
+      <c r="C5" s="82" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="19" t="s">
@@ -7287,8 +6738,8 @@
       <c r="E5" s="17"/>
     </row>
     <row r="6" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="85"/>
-      <c r="C6" s="88"/>
+      <c r="B6" s="80"/>
+      <c r="C6" s="83"/>
       <c r="D6" s="20" t="s">
         <v>4</v>
       </c>
@@ -7308,27 +6759,27 @@
       <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="76">
+      <c r="C9" s="84">
         <f>E5</f>
         <v>0</v>
       </c>
-      <c r="D9" s="77"/>
-      <c r="E9" s="78"/>
+      <c r="D9" s="85"/>
+      <c r="E9" s="86"/>
     </row>
     <row r="10" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="72"/>
-      <c r="D10" s="73"/>
+      <c r="C10" s="87"/>
+      <c r="D10" s="88"/>
       <c r="E10" s="23"/>
     </row>
     <row r="11" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="74"/>
-      <c r="D11" s="75"/>
+      <c r="C11" s="89"/>
+      <c r="D11" s="90"/>
       <c r="E11" s="23"/>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
@@ -7372,28 +6823,28 @@
       <c r="B25" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="76">
+      <c r="C25" s="84">
         <f>E5</f>
         <v>0</v>
       </c>
-      <c r="D25" s="77"/>
-      <c r="E25" s="78"/>
+      <c r="D25" s="85"/>
+      <c r="E25" s="86"/>
     </row>
     <row r="26" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="72"/>
-      <c r="D26" s="79"/>
-      <c r="E26" s="73"/>
+      <c r="C26" s="87"/>
+      <c r="D26" s="91"/>
+      <c r="E26" s="88"/>
     </row>
     <row r="27" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="74"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="75"/>
+      <c r="C27" s="89"/>
+      <c r="D27" s="92"/>
+      <c r="E27" s="90"/>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C29" s="21"/>
@@ -7431,18 +6882,18 @@
   <sheetData>
     <row r="1" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C2" s="81">
+      <c r="C2" s="76">
         <f>Summary!D26</f>
         <v>0</v>
       </c>
-      <c r="D2" s="82"/>
+      <c r="D2" s="77"/>
     </row>
     <row r="3" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="83" t="str">
+      <c r="B3" s="78" t="str">
         <f>Summary!B27</f>
         <v>06_Contact</v>
       </c>
-      <c r="C3" s="86" t="s">
+      <c r="C3" s="81" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="18" t="s">
@@ -7451,16 +6902,16 @@
       <c r="E3" s="17"/>
     </row>
     <row r="4" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="84"/>
-      <c r="C4" s="87"/>
+      <c r="B4" s="79"/>
+      <c r="C4" s="82"/>
       <c r="D4" s="19" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="17"/>
     </row>
     <row r="5" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="84"/>
-      <c r="C5" s="87" t="s">
+      <c r="B5" s="79"/>
+      <c r="C5" s="82" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="19" t="s">
@@ -7469,8 +6920,8 @@
       <c r="E5" s="17"/>
     </row>
     <row r="6" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="85"/>
-      <c r="C6" s="88"/>
+      <c r="B6" s="80"/>
+      <c r="C6" s="83"/>
       <c r="D6" s="20" t="s">
         <v>4</v>
       </c>
@@ -7490,26 +6941,26 @@
       <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="76">
+      <c r="C9" s="84">
         <f>E5</f>
         <v>0</v>
       </c>
-      <c r="D9" s="77"/>
-      <c r="E9" s="89"/>
+      <c r="D9" s="85"/>
+      <c r="E9" s="93"/>
     </row>
     <row r="10" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="72"/>
-      <c r="D10" s="73"/>
+      <c r="C10" s="87"/>
+      <c r="D10" s="88"/>
     </row>
     <row r="11" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="74"/>
-      <c r="D11" s="75"/>
+      <c r="C11" s="89"/>
+      <c r="D11" s="90"/>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C12" s="16"/>
@@ -7552,28 +7003,28 @@
       <c r="B25" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="76">
+      <c r="C25" s="84">
         <f>E5</f>
         <v>0</v>
       </c>
-      <c r="D25" s="77"/>
-      <c r="E25" s="78"/>
+      <c r="D25" s="85"/>
+      <c r="E25" s="86"/>
     </row>
     <row r="26" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="72"/>
-      <c r="D26" s="79"/>
-      <c r="E26" s="73"/>
+      <c r="C26" s="87"/>
+      <c r="D26" s="91"/>
+      <c r="E26" s="88"/>
     </row>
     <row r="27" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="74"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="75"/>
+      <c r="C27" s="89"/>
+      <c r="D27" s="92"/>
+      <c r="E27" s="90"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -7607,18 +7058,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C2" s="81">
+      <c r="C2" s="76">
         <f>Summary!D30</f>
         <v>0</v>
       </c>
-      <c r="D2" s="82"/>
+      <c r="D2" s="77"/>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B3" s="83" t="str">
+      <c r="B3" s="78" t="str">
         <f>Summary!B31</f>
         <v>07_Privacy</v>
       </c>
-      <c r="C3" s="86" t="s">
+      <c r="C3" s="81" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="18" t="s">
@@ -7627,16 +7078,16 @@
       <c r="E3" s="33"/>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B4" s="84"/>
-      <c r="C4" s="87"/>
+      <c r="B4" s="79"/>
+      <c r="C4" s="82"/>
       <c r="D4" s="19" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="35"/>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B5" s="84"/>
-      <c r="C5" s="87" t="s">
+      <c r="B5" s="79"/>
+      <c r="C5" s="82" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="19" t="s">
@@ -7645,8 +7096,8 @@
       <c r="E5" s="36"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B6" s="85"/>
-      <c r="C6" s="88"/>
+      <c r="B6" s="80"/>
+      <c r="C6" s="83"/>
       <c r="D6" s="20" t="s">
         <v>4</v>
       </c>
@@ -7666,27 +7117,27 @@
       <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="76">
+      <c r="C9" s="84">
         <f>E5</f>
         <v>0</v>
       </c>
-      <c r="D9" s="77"/>
-      <c r="E9" s="78"/>
+      <c r="D9" s="85"/>
+      <c r="E9" s="86"/>
     </row>
     <row r="10" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="72"/>
-      <c r="D10" s="73"/>
+      <c r="C10" s="87"/>
+      <c r="D10" s="88"/>
       <c r="E10" s="23"/>
     </row>
     <row r="11" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="74"/>
-      <c r="D11" s="75"/>
+      <c r="C11" s="89"/>
+      <c r="D11" s="90"/>
       <c r="E11" s="23"/>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
@@ -7718,28 +7169,28 @@
       <c r="B25" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="76">
+      <c r="C25" s="84">
         <f>E5</f>
         <v>0</v>
       </c>
-      <c r="D25" s="77"/>
-      <c r="E25" s="78"/>
+      <c r="D25" s="85"/>
+      <c r="E25" s="86"/>
     </row>
     <row r="26" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="72"/>
-      <c r="D26" s="79"/>
-      <c r="E26" s="73"/>
+      <c r="C26" s="87"/>
+      <c r="D26" s="91"/>
+      <c r="E26" s="88"/>
     </row>
     <row r="27" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="74"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="75"/>
+      <c r="C27" s="89"/>
+      <c r="D27" s="92"/>
+      <c r="E27" s="90"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -7773,18 +7224,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C2" s="81">
+      <c r="C2" s="76">
         <f>Summary!D34</f>
         <v>0</v>
       </c>
-      <c r="D2" s="82"/>
+      <c r="D2" s="77"/>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B3" s="83" t="str">
+      <c r="B3" s="78" t="str">
         <f>Summary!B35</f>
         <v>08_Game Testing</v>
       </c>
-      <c r="C3" s="86" t="s">
+      <c r="C3" s="81" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="18" t="s">
@@ -7793,16 +7244,16 @@
       <c r="E3" s="17"/>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B4" s="84"/>
-      <c r="C4" s="87"/>
+      <c r="B4" s="79"/>
+      <c r="C4" s="82"/>
       <c r="D4" s="19" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="17"/>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B5" s="84"/>
-      <c r="C5" s="87" t="s">
+      <c r="B5" s="79"/>
+      <c r="C5" s="82" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="19" t="s">
@@ -7811,8 +7262,8 @@
       <c r="E5" s="17"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B6" s="85"/>
-      <c r="C6" s="88"/>
+      <c r="B6" s="80"/>
+      <c r="C6" s="83"/>
       <c r="D6" s="20" t="s">
         <v>4</v>
       </c>
@@ -7832,27 +7283,27 @@
       <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="76">
+      <c r="C9" s="84">
         <f>E5</f>
         <v>0</v>
       </c>
-      <c r="D9" s="77"/>
-      <c r="E9" s="78"/>
+      <c r="D9" s="85"/>
+      <c r="E9" s="86"/>
     </row>
     <row r="10" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="72"/>
-      <c r="D10" s="73"/>
+      <c r="C10" s="87"/>
+      <c r="D10" s="88"/>
       <c r="E10" s="23"/>
     </row>
     <row r="11" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="74"/>
-      <c r="D11" s="75"/>
+      <c r="C11" s="89"/>
+      <c r="D11" s="90"/>
       <c r="E11" s="23"/>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
@@ -7896,28 +7347,28 @@
       <c r="B25" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="76">
+      <c r="C25" s="84">
         <f>E5</f>
         <v>0</v>
       </c>
-      <c r="D25" s="77"/>
-      <c r="E25" s="78"/>
+      <c r="D25" s="85"/>
+      <c r="E25" s="86"/>
     </row>
     <row r="26" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="72"/>
-      <c r="D26" s="79"/>
-      <c r="E26" s="73"/>
+      <c r="C26" s="87"/>
+      <c r="D26" s="91"/>
+      <c r="E26" s="88"/>
     </row>
     <row r="27" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="74"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="75"/>
+      <c r="C27" s="89"/>
+      <c r="D27" s="92"/>
+      <c r="E27" s="90"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -7937,6 +7388,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="851fd863-1f96-44b1-878a-247793b557e9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d55a6ab-b9f4-4be6-b06a-2cc46fdc62a1" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D539BB261075264EADE6FB64A6A44314" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f8545620b90e3ca3b4fa9c0eed4ef96d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="851fd863-1f96-44b1-878a-247793b557e9" xmlns:ns3="2d55a6ab-b9f4-4be6-b06a-2cc46fdc62a1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b2cedb268f8f7bfc874339ceeb7c9957" ns2:_="" ns3:_="">
     <xsd:import namespace="851fd863-1f96-44b1-878a-247793b557e9"/>
@@ -8165,41 +7636,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="851fd863-1f96-44b1-878a-247793b557e9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d55a6ab-b9f4-4be6-b06a-2cc46fdc62a1" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F5D0948-37AE-4A53-8E3A-E23AA9EDC499}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB6E2078-3560-474E-801B-A28E523CFF9F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="851fd863-1f96-44b1-878a-247793b557e9"/>
-    <ds:schemaRef ds:uri="2d55a6ab-b9f4-4be6-b06a-2cc46fdc62a1"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8222,9 +7662,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB6E2078-3560-474E-801B-A28E523CFF9F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F5D0948-37AE-4A53-8E3A-E23AA9EDC499}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="851fd863-1f96-44b1-878a-247793b557e9"/>
+    <ds:schemaRef ds:uri="2d55a6ab-b9f4-4be6-b06a-2cc46fdc62a1"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>